<commit_message>
RQ3 re-run with patched fault detection pipeline
</commit_message>
<xml_diff>
--- a/files/Cases/RQ3_Summary_EdgeOmission_ForPhDThesis.xlsx
+++ b/files/Cases/RQ3_Summary_EdgeOmission_ForPhDThesis.xlsx
@@ -486,19 +486,19 @@
         <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>91.3</v>
       </c>
       <c r="F2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G2" t="n">
-        <v>15.5</v>
+        <v>14</v>
       </c>
       <c r="H2" t="n">
-        <v>50</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="3">
@@ -618,7 +618,7 @@
         <v>20</v>
       </c>
       <c r="H6" t="n">
-        <v>35.26</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="7">
@@ -648,7 +648,7 @@
         <v>19</v>
       </c>
       <c r="H7" t="n">
-        <v>37.77</v>
+        <v>37.78</v>
       </c>
     </row>
     <row r="8">
@@ -675,7 +675,7 @@
         <v>44</v>
       </c>
       <c r="G8" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="H8" t="n">
         <v>40.91</v>
@@ -702,13 +702,13 @@
         <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>35</v>
+        <v>35.5</v>
       </c>
       <c r="G9" t="n">
         <v>16.5</v>
       </c>
       <c r="H9" t="n">
-        <v>46.96</v>
+        <v>47.22</v>
       </c>
     </row>
     <row r="10">
@@ -768,7 +768,7 @@
         <v>21.5</v>
       </c>
       <c r="H11" t="n">
-        <v>48.96</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -858,7 +858,7 @@
         <v>33.5</v>
       </c>
       <c r="H14" t="n">
-        <v>48.98</v>
+        <v>48.12</v>
       </c>
     </row>
     <row r="15">
@@ -915,7 +915,7 @@
         <v>320</v>
       </c>
       <c r="G16" t="n">
-        <v>29.25</v>
+        <v>30.25</v>
       </c>
       <c r="H16" t="n">
         <v>10</v>
@@ -942,13 +942,13 @@
         <v>100</v>
       </c>
       <c r="F17" t="n">
-        <v>122.5</v>
+        <v>112</v>
       </c>
       <c r="G17" t="n">
-        <v>26.25</v>
+        <v>24</v>
       </c>
       <c r="H17" t="n">
-        <v>18.35</v>
+        <v>22.66</v>
       </c>
     </row>
     <row r="18">
@@ -966,19 +966,19 @@
         <v>68</v>
       </c>
       <c r="D18" t="n">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>56.72</v>
       </c>
       <c r="F18" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="G18" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H18" t="n">
-        <v>20.49</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="19">
@@ -1005,10 +1005,10 @@
         <v>311</v>
       </c>
       <c r="G19" t="n">
-        <v>24</v>
+        <v>35.5</v>
       </c>
       <c r="H19" t="n">
-        <v>5.57</v>
+        <v>11.41</v>
       </c>
     </row>
     <row r="20">
@@ -1035,10 +1035,10 @@
         <v>404</v>
       </c>
       <c r="G20" t="n">
-        <v>24</v>
+        <v>35.5</v>
       </c>
       <c r="H20" t="n">
-        <v>3.65</v>
+        <v>8.789999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1065,10 +1065,10 @@
         <v>404</v>
       </c>
       <c r="G21" t="n">
-        <v>24</v>
+        <v>35.5</v>
       </c>
       <c r="H21" t="n">
-        <v>3.21</v>
+        <v>8.789999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -1086,19 +1086,19 @@
         <v>68</v>
       </c>
       <c r="D22" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E22" t="n">
-        <v>40.28</v>
+        <v>36.76</v>
       </c>
       <c r="F22" t="n">
         <v>282</v>
       </c>
       <c r="G22" t="n">
-        <v>21.75</v>
+        <v>22.5</v>
       </c>
       <c r="H22" t="n">
-        <v>7.55</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="23">
@@ -1116,19 +1116,19 @@
         <v>68</v>
       </c>
       <c r="D23" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E23" t="n">
-        <v>41.67</v>
+        <v>38.24</v>
       </c>
       <c r="F23" t="n">
         <v>391</v>
       </c>
       <c r="G23" t="n">
-        <v>21.25</v>
+        <v>21.5</v>
       </c>
       <c r="H23" t="n">
-        <v>4.65</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="24">
@@ -1146,19 +1146,19 @@
         <v>68</v>
       </c>
       <c r="D24" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E24" t="n">
-        <v>43.06</v>
+        <v>39.71</v>
       </c>
       <c r="F24" t="n">
         <v>507</v>
       </c>
       <c r="G24" t="n">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="H24" t="n">
-        <v>3.86</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="25">
@@ -1176,19 +1176,19 @@
         <v>68</v>
       </c>
       <c r="D25" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E25" t="n">
-        <v>100</v>
+        <v>95.83</v>
       </c>
       <c r="F25" t="n">
-        <v>769</v>
+        <v>618</v>
       </c>
       <c r="G25" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H25" t="n">
-        <v>2.58</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="26">
@@ -1206,19 +1206,19 @@
         <v>46</v>
       </c>
       <c r="D26" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E26" t="n">
-        <v>74.51000000000001</v>
+        <v>55.22</v>
       </c>
       <c r="F26" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G26" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="H26" t="n">
-        <v>42.33</v>
+        <v>31.82</v>
       </c>
     </row>
     <row r="27">
@@ -1278,7 +1278,7 @@
         <v>40</v>
       </c>
       <c r="H28" t="n">
-        <v>22.78</v>
+        <v>22.73</v>
       </c>
     </row>
     <row r="29">
@@ -1308,7 +1308,7 @@
         <v>46.5</v>
       </c>
       <c r="H29" t="n">
-        <v>14.04</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="30">
@@ -1338,7 +1338,7 @@
         <v>38</v>
       </c>
       <c r="H30" t="n">
-        <v>28.32</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="31">
@@ -1368,7 +1368,7 @@
         <v>49</v>
       </c>
       <c r="H31" t="n">
-        <v>24.42</v>
+        <v>24.46</v>
       </c>
     </row>
     <row r="32">
@@ -1398,7 +1398,7 @@
         <v>50</v>
       </c>
       <c r="H32" t="n">
-        <v>18.23</v>
+        <v>18.22</v>
       </c>
     </row>
     <row r="33">
@@ -1422,13 +1422,13 @@
         <v>100</v>
       </c>
       <c r="F33" t="n">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="G33" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H33" t="n">
-        <v>21.68</v>
+        <v>22.34</v>
       </c>
     </row>
     <row r="34">
@@ -1446,19 +1446,19 @@
         <v>6</v>
       </c>
       <c r="D34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" t="n">
         <v>100</v>
       </c>
       <c r="F34" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="G34" t="n">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="H34" t="n">
-        <v>58.12</v>
+        <v>53.57</v>
       </c>
     </row>
     <row r="35">
@@ -1575,7 +1575,7 @@
         <v>25</v>
       </c>
       <c r="G38" t="n">
-        <v>6.5</v>
+        <v>5.25</v>
       </c>
       <c r="H38" t="n">
         <v>31.74</v>
@@ -1605,10 +1605,10 @@
         <v>21</v>
       </c>
       <c r="G39" t="n">
-        <v>7.25</v>
+        <v>6.25</v>
       </c>
       <c r="H39" t="n">
-        <v>38.39</v>
+        <v>36.05</v>
       </c>
     </row>
     <row r="40">
@@ -1635,7 +1635,7 @@
         <v>16.5</v>
       </c>
       <c r="G40" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="H40" t="n">
         <v>43</v>
@@ -1686,19 +1686,19 @@
         <v>509.5</v>
       </c>
       <c r="D42" t="n">
-        <v>509.5</v>
+        <v>72</v>
       </c>
       <c r="E42" t="n">
-        <v>100</v>
+        <v>14.34</v>
       </c>
       <c r="F42" t="n">
-        <v>924</v>
+        <v>626</v>
       </c>
       <c r="G42" t="n">
-        <v>65</v>
+        <v>63.75</v>
       </c>
       <c r="H42" t="n">
-        <v>6.72</v>
+        <v>10.74</v>
       </c>
     </row>
     <row r="43">
@@ -1725,10 +1725,10 @@
         <v>2668</v>
       </c>
       <c r="G43" t="n">
-        <v>53</v>
+        <v>919.25</v>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>33.44</v>
       </c>
     </row>
     <row r="44">
@@ -1755,10 +1755,10 @@
         <v>3269</v>
       </c>
       <c r="G44" t="n">
-        <v>75</v>
+        <v>1043.25</v>
       </c>
       <c r="H44" t="n">
-        <v>2.4</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="45">
@@ -1785,10 +1785,10 @@
         <v>4867</v>
       </c>
       <c r="G45" t="n">
-        <v>80</v>
+        <v>1419.5</v>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>29.02</v>
       </c>
     </row>
     <row r="46">
@@ -1836,19 +1836,19 @@
         <v>509.5</v>
       </c>
       <c r="D47" t="n">
-        <v>509.5</v>
+        <v>32</v>
       </c>
       <c r="E47" t="n">
-        <v>100</v>
+        <v>6.78</v>
       </c>
       <c r="F47" t="n">
         <v>214</v>
       </c>
       <c r="G47" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="H47" t="n">
-        <v>7.56</v>
+        <v>30.14</v>
       </c>
     </row>
     <row r="48">
@@ -1866,19 +1866,19 @@
         <v>509.5</v>
       </c>
       <c r="D48" t="n">
-        <v>509.5</v>
+        <v>40</v>
       </c>
       <c r="E48" t="n">
-        <v>100</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="F48" t="n">
         <v>510</v>
       </c>
       <c r="G48" t="n">
-        <v>9</v>
+        <v>73.5</v>
       </c>
       <c r="H48" t="n">
-        <v>2.53</v>
+        <v>16.37</v>
       </c>
     </row>
     <row r="49">
@@ -1896,19 +1896,19 @@
         <v>509.5</v>
       </c>
       <c r="D49" t="n">
-        <v>509.5</v>
+        <v>400</v>
       </c>
       <c r="E49" t="n">
-        <v>100</v>
+        <v>83.88</v>
       </c>
       <c r="F49" t="n">
-        <v>96687.5</v>
+        <v>95712</v>
       </c>
       <c r="G49" t="n">
-        <v>271.5</v>
+        <v>5907</v>
       </c>
       <c r="H49" t="n">
-        <v>0.28</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="50">
@@ -1926,19 +1926,19 @@
         <v>36.5</v>
       </c>
       <c r="D50" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E50" t="n">
-        <v>87.88</v>
+        <v>24.32</v>
       </c>
       <c r="F50" t="n">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="G50" t="n">
-        <v>17.5</v>
+        <v>6</v>
       </c>
       <c r="H50" t="n">
-        <v>21.15</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="51">
@@ -1965,10 +1965,10 @@
         <v>160</v>
       </c>
       <c r="G51" t="n">
-        <v>19</v>
+        <v>19.75</v>
       </c>
       <c r="H51" t="n">
-        <v>11.39</v>
+        <v>11.95</v>
       </c>
     </row>
     <row r="52">
@@ -1995,10 +1995,10 @@
         <v>214</v>
       </c>
       <c r="G52" t="n">
-        <v>19</v>
+        <v>19.75</v>
       </c>
       <c r="H52" t="n">
-        <v>8.49</v>
+        <v>8.74</v>
       </c>
     </row>
     <row r="53">
@@ -2025,10 +2025,10 @@
         <v>214</v>
       </c>
       <c r="G53" t="n">
-        <v>19</v>
+        <v>19.75</v>
       </c>
       <c r="H53" t="n">
-        <v>8.49</v>
+        <v>8.609999999999999</v>
       </c>
     </row>
     <row r="54">
@@ -2046,19 +2046,19 @@
         <v>36.5</v>
       </c>
       <c r="D54" t="n">
-        <v>36.5</v>
+        <v>29</v>
       </c>
       <c r="E54" t="n">
-        <v>100</v>
+        <v>87.88</v>
       </c>
       <c r="F54" t="n">
         <v>446</v>
       </c>
       <c r="G54" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H54" t="n">
-        <v>6.77</v>
+        <v>4.89</v>
       </c>
     </row>
     <row r="55">
@@ -2076,19 +2076,19 @@
         <v>36.5</v>
       </c>
       <c r="D55" t="n">
-        <v>36.5</v>
+        <v>29</v>
       </c>
       <c r="E55" t="n">
-        <v>100</v>
+        <v>87.88</v>
       </c>
       <c r="F55" t="n">
         <v>554</v>
       </c>
       <c r="G55" t="n">
-        <v>34.75</v>
+        <v>26</v>
       </c>
       <c r="H55" t="n">
-        <v>5.68</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="56">
@@ -2106,19 +2106,19 @@
         <v>36.5</v>
       </c>
       <c r="D56" t="n">
-        <v>36.5</v>
+        <v>29</v>
       </c>
       <c r="E56" t="n">
-        <v>100</v>
+        <v>87.88</v>
       </c>
       <c r="F56" t="n">
         <v>703</v>
       </c>
       <c r="G56" t="n">
-        <v>36.75</v>
+        <v>26</v>
       </c>
       <c r="H56" t="n">
-        <v>4.88</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="57">
@@ -2142,13 +2142,13 @@
         <v>100</v>
       </c>
       <c r="F57" t="n">
-        <v>321.5</v>
+        <v>348</v>
       </c>
       <c r="G57" t="n">
-        <v>19.75</v>
+        <v>20</v>
       </c>
       <c r="H57" t="n">
-        <v>6.08</v>
+        <v>5.78</v>
       </c>
     </row>
     <row r="58">
@@ -2166,19 +2166,19 @@
         <v>19</v>
       </c>
       <c r="D58" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E58" t="n">
-        <v>78.95</v>
+        <v>58.82</v>
       </c>
       <c r="F58" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G58" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H58" t="n">
-        <v>50</v>
+        <v>39.47</v>
       </c>
     </row>
     <row r="59">
@@ -2208,7 +2208,7 @@
         <v>15</v>
       </c>
       <c r="H59" t="n">
-        <v>54.55</v>
+        <v>54.35</v>
       </c>
     </row>
     <row r="60">
@@ -2328,7 +2328,7 @@
         <v>13.5</v>
       </c>
       <c r="H63" t="n">
-        <v>44.83</v>
+        <v>46.55</v>
       </c>
     </row>
     <row r="64">
@@ -2358,7 +2358,7 @@
         <v>13</v>
       </c>
       <c r="H64" t="n">
-        <v>19.38</v>
+        <v>19.09</v>
       </c>
     </row>
     <row r="65">
@@ -2382,13 +2382,13 @@
         <v>100</v>
       </c>
       <c r="F65" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G65" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H65" t="n">
-        <v>24.12</v>
+        <v>27.42</v>
       </c>
     </row>
   </sheetData>
@@ -2535,16 +2535,16 @@
         <v>68</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>95.59</v>
       </c>
       <c r="F4" t="n">
         <v>740</v>
       </c>
       <c r="G4" t="n">
-        <v>19</v>
+        <v>35.5</v>
       </c>
       <c r="H4" t="n">
-        <v>2.64</v>
+        <v>4.63</v>
       </c>
     </row>
     <row r="5">
@@ -2622,19 +2622,19 @@
         <v>509.5</v>
       </c>
       <c r="D7" t="n">
-        <v>509.5</v>
+        <v>409</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>85.88</v>
       </c>
       <c r="F7" t="n">
         <v>97217</v>
       </c>
       <c r="G7" t="n">
-        <v>322</v>
+        <v>6038.5</v>
       </c>
       <c r="H7" t="n">
-        <v>0.34</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="8">
@@ -2958,19 +2958,19 @@
         <v>73</v>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>60.27</v>
       </c>
       <c r="F8" t="n">
         <v>45</v>
       </c>
       <c r="G8" t="n">
-        <v>20</v>
+        <v>23.5</v>
       </c>
       <c r="H8" t="n">
-        <v>44.44</v>
+        <v>52.22</v>
       </c>
     </row>
     <row r="9">
@@ -2988,19 +2988,19 @@
         <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>95.83</v>
       </c>
       <c r="F9" t="n">
         <v>618</v>
       </c>
       <c r="G9" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H9" t="n">
-        <v>2.91</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="10">
@@ -3027,10 +3027,10 @@
         <v>869</v>
       </c>
       <c r="G10" t="n">
-        <v>19</v>
+        <v>35.5</v>
       </c>
       <c r="H10" t="n">
-        <v>2.12</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="11">
@@ -3228,19 +3228,19 @@
         <v>509.5</v>
       </c>
       <c r="D17" t="n">
-        <v>509.5</v>
+        <v>365</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>74.06999999999999</v>
       </c>
       <c r="F17" t="n">
         <v>53452</v>
       </c>
       <c r="G17" t="n">
-        <v>361</v>
+        <v>3244</v>
       </c>
       <c r="H17" t="n">
-        <v>0.68</v>
+        <v>7.02</v>
       </c>
     </row>
     <row r="18">
@@ -3258,19 +3258,19 @@
         <v>509.5</v>
       </c>
       <c r="D18" t="n">
-        <v>509.5</v>
+        <v>400</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>83.88</v>
       </c>
       <c r="F18" t="n">
         <v>95712</v>
       </c>
       <c r="G18" t="n">
-        <v>369</v>
+        <v>5907</v>
       </c>
       <c r="H18" t="n">
-        <v>0.35</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="19">
@@ -3288,19 +3288,19 @@
         <v>509.5</v>
       </c>
       <c r="D19" t="n">
-        <v>509.5</v>
+        <v>455</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>91.91</v>
       </c>
       <c r="F19" t="n">
         <v>173964</v>
       </c>
       <c r="G19" t="n">
-        <v>256</v>
+        <v>9022</v>
       </c>
       <c r="H19" t="n">
-        <v>0.13</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="20">

</xml_diff>